<commit_message>
Salvataggio file residui: organigramma, komunigo-ordine/v14, import-fornitori, schema-v121
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/organigramma/organigramma-dati_1.xlsx
+++ b/organigramma/organigramma-dati_1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{1EF0A91C-2001-4783-AA0A-BF634189E4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96F2C3E3-BB0F-4FEC-B67D-DA166D2B2C36}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{1EF0A91C-2001-4783-AA0A-BF634189E4C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69990E77-0369-4841-A8E3-6606CDE883B9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,12 +12,25 @@
     <sheet name="Liste" sheetId="2" r:id="rId2"/>
     <sheet name="Istruzioni" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="101">
   <si>
     <t>ORGANIGRAMMA — compila una riga per persona</t>
   </si>
@@ -190,9 +203,6 @@
     <t xml:space="preserve">rapporto con i grandi clienti </t>
   </si>
   <si>
-    <t>gestione ordini clienti e fornitori; Inserimento ordini clienti e fornitori; ricerca materiali</t>
-  </si>
-  <si>
     <t>Vito Barbara</t>
   </si>
   <si>
@@ -256,9 +266,6 @@
     <t>allestitore interno</t>
   </si>
   <si>
-    <t>allestimento cartotecnica, tipografia e digitale; aiuto nei reparti che hanno bisono</t>
-  </si>
-  <si>
     <t>Incisione Telai; recupero e sviluppo telai; stampa serigrafica; stampa digitale; allestimenti interni; lavorazioni con la pressa; aiuto nei reparti che hanno bisogno</t>
   </si>
   <si>
@@ -268,15 +275,9 @@
     <t>Magazziniere</t>
   </si>
   <si>
-    <t>Bo</t>
-  </si>
-  <si>
     <t>carico e scarico merci; preparazione ordini; sistemazione materiale eventi; gestione materiali interni di consumo</t>
   </si>
   <si>
-    <t>non lo so</t>
-  </si>
-  <si>
     <t>Julio Landaverde</t>
   </si>
   <si>
@@ -298,16 +299,40 @@
     <t>Allestitore / Fresatore</t>
   </si>
   <si>
-    <t>lavorazioni cnc; allestimento interno e esterno</t>
-  </si>
-  <si>
     <t>Lica Popa</t>
   </si>
   <si>
-    <t>Autista / Allestitore</t>
-  </si>
-  <si>
-    <t>ritiri e consegne; allestimento interno e esterno; manutentore stabile interno e esterno;</t>
+    <t>gestione ordini clienti; Inserimento ordini clienti; ricerca materiali</t>
+  </si>
+  <si>
+    <t>gestione ordini fornitori; Inserimento ordini fornitori; controllo fatture; negoziare fornitore</t>
+  </si>
+  <si>
+    <t>Andrea Bonanni/Kledi Dell'Omo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modellazione 3D; Progettazione strutture e stand; Sviluppo grafiche; Rendering; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebecca Bertilone </t>
+  </si>
+  <si>
+    <t>allestimento cartotecnica, tipografia e digitale; aiuto nei reparti che hanno bisogno</t>
+  </si>
+  <si>
+    <t>Cristina Mammetti; Vito Barbara</t>
+  </si>
+  <si>
+    <t>lavorazioni cnc; allestimento interno e esterno; impianti elettrici</t>
+  </si>
+  <si>
+    <t>allestimento interno e esterno; manutentore stabile interno e esterno; ritiri e consegne;</t>
+  </si>
+  <si>
+    <t>Allestitore / Autista</t>
+  </si>
+  <si>
+    <t>Allestimento</t>
   </si>
 </sst>
 </file>
@@ -433,6 +458,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -884,7 +913,7 @@
         <v>53</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>16</v>
@@ -911,7 +940,7 @@
         <v>54</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>16</v>
@@ -920,10 +949,10 @@
         <v>55</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>17</v>
@@ -935,10 +964,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>16</v>
@@ -947,7 +976,7 @@
         <v>54</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>57</v>
+        <v>91</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>54</v>
@@ -962,19 +991,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>64</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>55</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>49</v>
@@ -989,22 +1018,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="E11" s="5" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>12</v>
@@ -1016,22 +1045,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>70</v>
-      </c>
       <c r="D12" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F12" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>72</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>12</v>
@@ -1043,22 +1072,22 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="G13" s="5" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>17</v>
@@ -1070,22 +1099,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>75</v>
-      </c>
       <c r="E14" s="5" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>12</v>
@@ -1097,22 +1126,22 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>78</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>59</v>
+        <v>92</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>12</v>
@@ -1124,22 +1153,22 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>24</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>12</v>
@@ -1151,22 +1180,22 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>90</v>
-      </c>
       <c r="G17" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>12</v>
@@ -1178,22 +1207,22 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>21</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>49</v>
+        <v>92</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>12</v>
@@ -1205,19 +1234,23 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D19" s="5"/>
+        <v>99</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="E19" s="5" t="s">
         <v>54</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="G19" s="5"/>
+        <v>98</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>79</v>
+      </c>
       <c r="H19" s="5" t="s">
         <v>12</v>
       </c>

</xml_diff>